<commit_message>
feat: direct upload-ready Excel (.xlsx) export strictly adhering to SmartBiz bulk_upload_template worksheet structure and 3-sheet workbook
</commit_message>
<xml_diff>
--- a/smartbiz_bulk_upload_template_v10.xlsx
+++ b/smartbiz_bulk_upload_template_v10.xlsx
@@ -7661,7 +7661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ56"/>
+  <dimension ref="A1:AZ1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="19.5" customWidth="1" min="1" max="1"/>
@@ -7973,3721 +7973,61 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="51" customHeight="1">
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>whl239_73330_rng_stn_om_12</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Om Mandala Rangoli Design – Mess-Free Pooja Decoration</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>539</v>
-      </c>
-      <c r="I2" t="n">
-        <v>259</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Enhance your pooja room or home entrance with this Om Mandala Rangoli design stencil. Perfect for creating a sacred and serene atmosphere during festivals and rituals, this stencil helps you achieve a clean, precise, and mess-free rangoli every time. Key features Sacred Om Design – Ideal for mandir, pooja rooms, and festive celebrations. Mess-Free Application – Keeps colors neatly within the stencil for crisp lines. Heavy MDF Base – Ensures stability and prevents movement even under a fan. Reusable and Durable – Made to last with sturdy materials for repeated use. Easy Maintenance – Simply brush off colors after use and store for next time. Materials &amp;amp; care Crafted from durable MDF, this rangoli stencil is designed for steady use. To maintain its quality, gently brush off any residual powd&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/nG8pP6034D.jpg</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/qjVOzEOdV6.jpg</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/7MiafrLHU9.jpg</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/eC4r57kdI4.jpg</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Wjirk4ymqK.jpg</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/9c038ad8-5546-4b2d-9475-6d6ce7435c04.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="51" customHeight="1">
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>whl313_90633_pm105_murti</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Panchmukhi Hanuman Idol for Home, Office &amp; Car Dashboard Spiritual Decor</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>499</v>
-      </c>
-      <c r="I3" t="n">
-        <v>349</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the divine presence of a Panchmukhi Hanuman idol , perfect for enhancing your spiritual space. This beautifully crafted idol embodies protection, courage, and devotion, bringing positive energy to your home, office, or car dashboard. Its intricate design and antique bronze finish make it a truly special addition to any decor. Key features Premium antique bronze finish with detailed craftsmanship Depicts the powerful Panchmukhi (Five-Faced) Hanuman form Symbol of protection, courage, devotion, and success Intricate traditional design with sacred weapons and ornaments Ideal for home temples, offices, and spiritual spaces Durable and elegant decorative idol Perfect gift for Hanuman Jayanti, Diwali, housewarming ceremonies, and religious occasions Materials &amp;amp; care Crafted with a durab&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/0fKCWS2Oce.jpg</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/P7wd9B2NAL.jpg</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/n8Y1s6GVMm.jpg</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4eGHmZINcF.jpg</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/lVdyq9JuSj.jpg</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/HH9yyt2nK9.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="51" customHeight="1">
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>whl239_73363_decor_laxmi_charan_paduka_s</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Laxmi Charan Paduka Stickers – Festive Spiritual Home Décor (Pack of 2)</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>559</v>
-      </c>
-      <c r="I4" t="n">
-        <v>229</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Enhance your home&amp;#x27;s spiritual aura with our Laxmi Charan Paduka Sticker Set, designed to bring blessings and prosperity during festivals and daily pooja rituals. These sacred Laxmi Charan Paduka stickers feature traditional footprints embellished with vibrant beads and sparkling stones for a divine touch, making them perfect for festive spiritual home decor. Key features Traditional Goddess Lakshmi footprints featuring the auspicious Swastik symbol Decorated with multicolored beads, sequins, and glittering stones for vibrant appeal Easy peel-and-stick backing suitable for doors, walls, floors, and pooja thalis Reusable and simple to clean with a dry wipe, ideal for multiple festive occasions Perfect for Diwali, Lakshmi Pujan, Navratri, Griha Pravesh, and spiritual home decoration Comes pac&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/01_9da764a6-0ee2-4da6-aac6-e8bc7849da42.jpg</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_d891c284-8708-4c38-b0e4-aeca264c3244.jpg</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_edf02a26-c1a5-4ee0-a634-cb9843a6d666.jpg</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_155b0a2f-27c8-4248-af67-d5b57806a5a7.jpg</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_1e5c06fe-75d5-4c51-afe2-d262f4fccc14.jpg</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/06_7f2a7e37-7e1e-4011-af4f-c64f39073aa9.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="51" customHeight="1">
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>9041_small_hand_tally_counter</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Hand Tally Counter for Jaap and Mantra Chanting Pooja Use</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>509</v>
-      </c>
-      <c r="I5" t="n">
-        <v>219</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;A digital finger tally counter with strap simplifies your spiritual practices by accurately tracking repetitions. This essential tool ensures your focus remains on your jaap or mantra chanting, removing the distraction of manual counting. Its compact design and comfortable strap make it ideal for extended use during daily prayers, meditation, or temple visits. Key features Keeps precise count for uninterrupted chanting and meditation One-thumb press operation allows for easy, discreet counting Reading holds even when paused, perfect for intermittent use Quick reset dial returns count to zero for new sessions Compact size with a strap for comfortable, secure wear on finger Manual click mechanism means no batteries are required Portable design fits easily in pooja thali, pocket, or bag Versa&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/9041_656ca080-9177-4b35-93ae-60b7732d45e4.png</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/eedc839b-60ab-46ad-99d2-45ecaa0c38f3.jpg</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/7_7da8be7e-c7e8-48ac-90bb-dd94e795c570.jpg</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/8_4ba63586-6093-450c-8983-0bb4ad8820ff.jpg</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/4_11d433d1-4d76-44b8-b5fa-30b7cf078440.jpg</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/5_62ec6240-78d3-49c8-902a-1c574b5f8eac.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="51" customHeight="1">
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>22198_hand_shape_kankavati_kumkum_holder</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Hand Shaped Kankavati – Elegant Puja Storage with Enamel Work</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>535</v>
-      </c>
-      <c r="I6" t="n">
-        <v>229</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the beauty and utility of the Hamsa hand decorative puja thali, an exquisite accessory designed for your sacred rituals. Crafted in a traditional hand (hamsa) shape, this kumkum holder features twin compartments for storing kumkum (roli) and chawal (rice), along with two additional lidded boxes for extra storage. Enhanced with intricate blue and teal enamel floral work on a rich golden finish, it adds a divine touch to your home temple, pooja thali, or festival celebrations. This elegant piece not only serves as a practical puja item but also accentuates the spiritual ambiance of your worship space. Key features Hamsa hand shaped decorative kumkum holder Dual compartments for kumkum and chawal Two extra lidded boxes for additional storage Rich golden finish with detailed enamel wo&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22198-01-no-sku_238ab33d-25cc-4182-82c4-47ef051b6e42.jpg</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22198-02-sku_b70a011f-7333-4e61-b427-3a05d88bfd4b.jpg</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22198-03-product_db2e4ff7-43b1-4168-ace1-6b2631e96070.jpg</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22198-04-product_c0d57e72-f3c9-4144-b5cb-d010ce441491.jpg</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22198-05-white-bg_27048fdf-a731-4c2b-a9a4-734b7cda6d2c.jpg</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22198-06-size_d81be685-bb60-4de5-b054-f198156a3229.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="51" customHeight="1">
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>whl175_94317_7104</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Decorative Palm Shape Ganesh Idols for Pooja Mandir, Table &amp; Home Decor (Set of 4)</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>479</v>
-      </c>
-      <c r="I7" t="n">
-        <v>349</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Add a distinctive devotional touch to your space with these Palm Shape Ganesh Idols. Each piece features Lord Ganesh seated within a hand-shaped frame, enhanced with metallic detailing that gives the idols a refined and traditional appearance. The compact design makes them suitable for home mandirs, pooja shelves, office desks, side tables and festive arrangements. The different metallic accents add variety while maintaining a coordinated overall look. Key Features Unique palm-shaped Ganesh idol design Decorative metallic detailing Elegant white finish Suitable for mandir and pooja setup Compact design for table and shelf placement Ideal for festive and devotional decoration Can be displayed together or separately Quantity: Set of 4&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/FxXtgzeQJm.png</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/ioyZy5nIog.png</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/s9wUTME51k.png</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/r91BKyN07e.png</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/zDQ0S1HOvP.png</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Kc9dgHYt5a.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="51" customHeight="1">
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2234_silver_bajot</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Aluminium Foil Bajot – Handcrafted Pooja Chowki for Home | Styleva</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>500</v>
-      </c>
-      <c r="I8" t="n">
-        <v>219</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Elevate your spiritual space and home aesthetics with our exquisite Aluminium Foil Bajot . This beautifully handcrafted pooja chowki is designed to add a touch of traditional elegance to your rituals and interior decor. Perfect for royal weddings, daily pujas, or as a charming accent piece, this versatile patla combines durability with a luxurious finish, making it an essential addition to any Indian home. Key features Luxurious Minakari Design: Adorned with intricate white metal minakari work over aluminium foil, creating a royal and eye-catching appearance. Sturdy Wooden Construction: Built on a solid wooden base for lasting durability and stability. Multipurpose Utility: Ideal for placing deity idols during pooja, sitting comfortably for rituals, or as a decorative stand for plants and&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/2_bdb9a21a-cd11-4af6-a6c7-f54b76dc16b9.jpg</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/2234SKUCODE.jpg</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/944879d7-32b1-4582-9b5a-83f6ced20d26.jpg</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/22341.jpg</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/4_2803ea4c-8890-4014-a2e1-9326a35f17ec.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="51" customHeight="1">
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>19675_shubh_labh_wall_hangings_2pc_no7</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Shubh Labh Wall Hangings – Set of 2 Festive Decorative Pieces</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>575</v>
-      </c>
-      <c r="I9" t="n">
-        <v>229</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Invite prosperity and good fortune into your home with this exquisite Shubh Labh wall hangings set. This vibrant set of two decorative pieces features traditional &amp;quot;Shubh&amp;quot; (auspicious) and &amp;quot;Labh&amp;quot; (profit) inscriptions, beautifully enhanced with shimmering glitter and intricate stonework. Perfect for elevating festive vibes or adding spiritual charm to your living spaces, these lightweight wall hangings instantly bring positivity and traditional Indian elegance. Key features Auspicious inscriptions: Displays &amp;quot;Shubh&amp;quot; and &amp;quot;Labh&amp;quot; symbols, promoting good luck and success. Festive design: Glitter-embellished and stone-studded for an eye-catching decorative appeal. Versatile placement: Ideal for home entrances, pooja rooms, temples, shops, or offices. Lightweight and easy to hang: Quick to install&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/01_8e3fcd8e-cfe6-4b3b-ad8e-780f5014fd5d.jpg</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/85c9a601-5322-428e-8145-60f1125d9a86.jpg</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_a36c43ec-b2ae-43ae-b6f3-4d0b7379be99.jpg</t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_65960b96-d73c-4105-a152-bbdaa8429caf.jpg</t>
-        </is>
-      </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_a4e5998b-cba0-46cd-99ea-494709aeea51.jpg</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_a27e5163-97d3-490d-a3e2-80709a0433ce.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="51" customHeight="1">
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>8444_led_iceberg_light_1pc</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Iceberg Night Light – Flameless LED Decor for Home | Indo Glow</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>460</v>
-      </c>
-      <c r="I10" t="n">
-        <v>259</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Transform your living space with the enchanting LED light-up clear iceberg decor from Indo Glow. This modern and unique flameless LED lamp creates a serene ambiance, perfect for any room. Ideal for bedroom decor, festive celebrations like Diwali, or as a thoughtful gift, its captivating iceberg design adds a touch of contemporary elegance without the hazards of traditional candles. Experience the perfect blend of style and safety with our innovative LED light-up clear iceberg decor. Powered by energy-efficient LEDs, it offers a gentle, calming glow that enhances your home&amp;#x27;s atmosphere. Whether you&amp;#x27;re looking to create a cozy reading nook, a tranquil bedroom sanctuary, or a festive display for special occasions, this versatile night light is an excellent choice. Its compact size makes it a&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/8444_led_iceberg_light_1pc.jpg</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/0ee593c4-95b9-4def-87cf-594eb2310c96.jpg</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/19417.png</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/19418.png</t>
-        </is>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/011_8d4ae56c-5560-44b2-8f46-e4f7fefbdcb2.jpg</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/2092621834.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="51" customHeight="1">
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>whl167_48605_handcrafted_tulsi_diya_4pc</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Handcrafted Tulsi Kiyaro Diya Set – Festive Clay Oil Lamps with Swastik &amp; Shree</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>459</v>
-      </c>
-      <c r="I11" t="n">
-        <v>299</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Celebrate your festivals with the Handcrafted Tulsi Kiyaro Diya Set, a perfect blend of tradition and vibrant decor. These clay oil lamps, adorned with sacred Swastik and Shree symbols, bring divine positivity and an auspicious atmosphere to your home. Ideal for Diwali, Navratri, Ganesh Chaturthi, weddings, and daily pooja rituals, these square-shaped diyas are a beautiful spiritual addition to your festive decor. Key features Hand-painted square diyas featuring sacred Hindu symbols like Swastik and Shree for spiritual significance. Made from high-quality clay that enhances traditional authenticity and durability. Multi-color palette including red, green, purple, and orange to brighten your festive ambiance. Compatible with oil, ghee, or tealight candles for versatile use. Eco-friendly and&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/cisTqUbngf.jpg</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Ae6zk3JnnF.jpg</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/10ax8Rhryi.jpg</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/pDAthNJ4UE.jpg</t>
-        </is>
-      </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/pZtERD6xxD.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="51" customHeight="1">
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>whl202_67906_diya_flower_5l_red</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Flower 5-Step Decorative Diya – Multi-Purpose Eco-Friendly Holder</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>480</v>
-      </c>
-      <c r="I12" t="n">
-        <v>249</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Festive &amp; Lights</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Enhance your home ambiance with the Flower 5-Step Decorative Diya, a versatile eco-friendly gypsum holder perfect for pooja rituals, festive lighting, or stylish decor. This multi-purpose diya blends traditional charm with modern functionality to illuminate your space with warmth and serenity. Key features Crafted from premium-quality, non-toxic, and durable gypsum, ensuring an eco-friendly product Intricately handcrafted lotus flower design symbolizing purity and peace Multi-use as a diya, tealight candle holder, dhoop cone stand, mini planter, or creative craft base Elegant and smooth finish complements pooja rooms, offices, living areas, and festive decorations Perfect for Diwali, Navratri, weddings, housewarmings, and gifting Customizable surface — easily painted or decorated to suit y&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/mOff8nPgzy.png</t>
-        </is>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/b456Ff1Wkc.png</t>
-        </is>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/uLHCbmbvTd.png</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/ZgWdJBsnmE.png</t>
-        </is>
-      </c>
-      <c r="AA12" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/vju4NtPzlL.png</t>
-        </is>
-      </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/x1aApIbqsH.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="51" customHeight="1">
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>10314_ss_kitchen_veg_n_friut_grater</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Stainless Steel Cheese Grater – Multi-Purpose Kitchen Tool | CookAura</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>550</v>
-      </c>
-      <c r="I13" t="n">
-        <v>229</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Elevate your culinary experience with the CookAura Stainless Steel Cheese Grater , an essential multi-purpose tool for every Indian kitchen. This versatile grater is designed to make food preparation quicker, easier, and more efficient, whether you&amp;#x27;re grating hard cheeses, shredding fresh vegetables, or zesting citrus fruits. Its durable construction and ergonomic design ensure a comfortable grip and superior performance for all your grating needs. Crafted from high-quality stainless steel, this kitchen essential promises long-lasting sharpness and resistance to rust, making it a reliable companion for years to come. From ginger and garlic to chocolate and potatoes, this efficient kitchen tool handles a wide array of ingredients with ease. Its compact design also ensures it won&amp;#x27;t take up m&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_b3320453-ee8d-4bf5-b0ea-623fe797673d.jpg</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_cd98e4a7-fd75-4603-8071-6ab9c25a5b02.jpg</t>
-        </is>
-      </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_dcc8733f-c840-45a9-8f09-c98c74856e3d.jpg</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/06_07060837-ddc5-4743-b877-f8f3a50a3c73.jpg</t>
-        </is>
-      </c>
-      <c r="AA13" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_c8bec7f9-6ccb-41a1-b3df-59122766b82b.jpg</t>
-        </is>
-      </c>
-      <c r="AB13" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/07_e6461edb-bfed-45f3-87cb-42e6adc0fb96.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="51" customHeight="1">
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2996_round_sili_strainer_1pc_no1</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Silicone Collapsible Strainer – Space-Saving Kitchen Tool for Easy Draining</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>519</v>
-      </c>
-      <c r="I14" t="n">
-        <v>319</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The silicone collapsible strainer is an essential kitchen accessory that simplifies draining and rinsing tasks. Its flexible, food-grade silicone body folds flat, allowing for compact storage while providing a sturdy, reliable strainer when needed. Designed for versatile use, this collapsible colander is perfect for washing fruits, vegetables, and rice, as well as draining pasta, noodles, and boiled foods. Its lightweight construction and easy-clean surface make it an ideal tool for busy kitchens, outdoor cooking, or travel. Key features Collapsible design folds flat for space-efficient storage Made of durable, food-grade silicone material Fine drain holes for quick, mess-free draining Comfortable side handles for secure grip Sturdy structure when popped up for rinsing Suitable for washing&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Silicone-Colander_2_-1.jpg</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/sku_52a6813f-0bcb-4dd1-9fcc-48c2d3628c0f.jpg</t>
-        </is>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Silicone-Colander_2_-3.jpg</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Silicone-Colander_2_-4.jpg</t>
-        </is>
-      </c>
-      <c r="AA14" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Silicone-Colander_2_-7.jpg</t>
-        </is>
-      </c>
-      <c r="AB14" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Silicone-Colander_2_-6.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="51" customHeight="1">
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>11401_plastic_gas_stove_burner_cover_10p</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Plastic Gas Stove Burner Cover Liners for Kitchen Cleaning and Hygiene (10 Pc)</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>480</v>
-      </c>
-      <c r="I15" t="n">
-        <v>349</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Disposable Plastic Gas Stove Burner Cover Liners with Raised Edges for Catching Oil, Food Spills and Cooking Residue Around Kitchen Burners (10 Pc) Description :- These gas stove burner cover liners help keep the cooking area cleaner by collecting oil splashes, food spills and residue around the burner. Their round open-center design fits around compatible stove burners and supports quicker cleanup during regular kitchen use. Key Features :- Open-center design fits around compatible gas burners Raised edges help contain spills and cooking residue Protective liner reduces direct mess on the stove surface Lightweight construction allows convenient placement Round shape provides practical burner-area coverage Disposable format supports quick cleanup after use Stackable design allows compact k&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/11401-1.jpg</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/11401-2.jpg</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/11401-3.jpg</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/11401-4.jpg</t>
-        </is>
-      </c>
-      <c r="AA15" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/11401-5.jpg</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/11401-6.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="51" customHeight="1">
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>5871_soup_spoon_long_handle</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Silicone Soup Spoon – Multifunctional Strainer &amp; Ladle | Quickslice</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>595</v>
-      </c>
-      <c r="I16" t="n">
-        <v>229</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Elevate your Indian kitchen experience with our premium Silicone Soup Spoon , designed for both efficiency and durability. This versatile kitchen tool is perfect for effortlessly serving soups, gravies, and stews, while its integrated straining function makes it ideal for separating liquids from solids. Crafted from high-quality, food-grade silicone with a robust stainless steel core, this long handle spoon ensures a comfortable grip and safe use on all types of cookware, including delicate non-stick surfaces. Say goodbye to scratched pots and hello to seamless cooking with Quickslice. Key features Food-Grade Silicone: Made from premium, BPA-free, and heat-resistant silicone, ensuring safety and longevity in your kitchen. Integrated Strainer: Cleverly designed with a perforated head, allow&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/5871_soup_spoon_long_handle.jpg</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/0ed09443-014e-4d3b-9487-75d14c668891_8053bb08-02de-45ca-8639-b2465cfb357a.jpg</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_88bfeeeb-59ec-4b83-972a-5c0f071e922c.jpg</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_2056ab04-47f2-45bd-959c-cb027f30e827.jpg</t>
-        </is>
-      </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_faae6e8c-cf16-4787-9417-9702bb7038d0.jpg</t>
-        </is>
-      </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_e328dddc-891e-47d3-b5a2-77d55b9dd450.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="51" customHeight="1">
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>whl282_21022_cute_teddy_bear_kids_water_</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Kids Water Bottle – Cartoon Bear Shape with Straw &amp; Strap</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>465</v>
-      </c>
-      <c r="I17" t="n">
-        <v>269</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Kids water bottle designed with a cute cartoon bear shape, featuring a built-in straw and shoulder strap to make hydration fun and easy for children. This kids water bottle encourages regular drinking with its leakproof flip-lock lid and transparent body to monitor water levels. Key features Fun cartoon bear design tailored for kids Convenient built-in straw for easy sipping Leakproof flip-lock lid prevents spills and leaks Adjustable shoulder strap for hands-free carrying Transparent body to easily check remaining water Lightweight and safe edges suitable for children Encourages kids to drink water regularly Perfect for school, travel, and outdoor activities Materials &amp;amp; care Made from high-quality plastic materials, this water bottle is easy to clean and maintain. Hand wash recommended to&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Bottle-01_8f4648a9-b2f8-43d1-9988-fe2d06cd44b5.jpg</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/8548082b-cecd-4ecc-a779-d0e2094031b7.jpg</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Bottle-04_a6b8d7f6-d411-461a-8ad2-075562f1f480.jpg</t>
-        </is>
-      </c>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/21022_cute_teddy_bear_kids_water_bottle_1pc.jpg</t>
-        </is>
-      </c>
-      <c r="AA17" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Bottle-05_79b91998-a4bf-4012-8ff4-a41f7297f602.jpg</t>
-        </is>
-      </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Bottle-06_81ae6ef2-c4f1-42a0-a098-64e3de016b31.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="51" customHeight="1">
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>5834_3in1_chopping_board_peeler_knife_se</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Kitchen Knife Set – 3 in 1 Knife, Chopping Board &amp; Peeler</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>460</v>
-      </c>
-      <c r="I18" t="n">
-        <v>269</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Experience the convenience of our Kitchen Knife Set, a versatile 3 in 1 solution featuring a sharp kitchen knife, sturdy chopping board, and an efficient vegetable peeler. Designed for easy and safe food prep, this set is perfect for slicing, chopping, and peeling fruits and vegetables effortlessly. Key features Includes a sharp kitchen knife for precise cutting Durable chopping board offering a stable, hygienic surface Vegetable peeler that makes peeling quick and easy Compact and lightweight design ideal for daily cooking Easy to clean and maintain for long-lasting use Perfect for home cooks and professional chefs alike FAQ Q1: What does the Kitchen Knife Set include? A: The set includes a sharp knife, a sturdy chopping board, and a vegetable peeler. Q2: Is this set suitable for daily us&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/36_chopping-board.jpg</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/sku_e97e52a4-ffc2-403f-b1f1-0a43a08c732b.jpg</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/35_chopping-board.jpg</t>
-        </is>
-      </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/38_chopping-board.jpg</t>
-        </is>
-      </c>
-      <c r="AA18" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/39_chopping-board.jpg</t>
-        </is>
-      </c>
-      <c r="AB18" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/43_chopping-board.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="51" customHeight="1">
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>10595_supermom_full_round_pincer</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Stainless Steel Full Round Kitchen Pincer – Heavy Duty Grip</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>485</v>
-      </c>
-      <c r="I19" t="n">
-        <v>329</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The stainless steel full round kitchen pincer offers heavy-duty, rust-resistant performance for safely handling hot cookware in any kitchen setting. Crafted from premium stainless steel, this kitchen pincer delivers unmatched durability and heat resistance, making it ideal for lifting and moving hot utensils like pressure cooker lids, kadhai, and tandoor grillware without risking burns. Its full round gripping ends provide a secure, slip-resistant hold, increasing safety and control with every use. Key features Made from premium stainless steel ensuring rust and corrosion resistance Full round gripping ends for firm, secure handling of hot cookware Ergonomic, slip-resistant handle for comfortable grip during extended use Heavy-duty construction supports lifting heavy pots and pans with eas&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/10595.png</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/sku_2b373ef3-c1de-43b4-8a05-afe9d3c70f0e.jpg</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/01_2cc68044-cd07-47c6-afc6-da5ce039f4b3.jpg</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_f817ef22-e426-45b7-b8ed-73be3d1d2eec.jpg</t>
-        </is>
-      </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_488e2cd9-49dc-4aed-9de6-cb7433861b80.jpg</t>
-        </is>
-      </c>
-      <c r="AB19" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_9ac277ac-4dd4-43c7-96cc-ecdd7bb572a6.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="51" customHeight="1">
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>10597_supermom_spring_o_masher</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Stainless Steel Potato Masher – Heavy Duty with Comfortable Grip</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>529</v>
-      </c>
-      <c r="I20" t="n">
-        <v>349</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The stainless steel potato masher is a heavy-duty kitchen essential designed for effortless mashing of vegetables, potatoes, and fruits. Featuring a robust spring design and ergonomic non-slip handle, this masher ensures smooth, even pressure for the perfect mash every time. Whether preparing mashed potatoes, pav bhaji, soups, or baby food, this kitchen masher delivers reliable performance for home cooks and professionals alike. Key features Durable stainless steel spring design offers long-lasting strength and efficient mashing. Ergonomic handle with a comfortable, non-slip grip for ease of use and better control. Perfect for mashing potatoes, vegetables, fruits, pav bhaji, soups, and baby food. Easy to clean and maintain for everyday kitchen tasks. Compact, lightweight design allows conv&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Maser-01.jpg</t>
-        </is>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/sku_88888870-0e35-41de-9966-35da992a8f27.jpg</t>
-        </is>
-      </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Maser-02.jpg</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Maser-03.jpg</t>
-        </is>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Maser-05.jpg</t>
-        </is>
-      </c>
-      <c r="AB20" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Maser-04.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="51" customHeight="1">
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>24591_vegetables_n_fruit_peeler_1pc</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Stainless Steel Vegetable and Fruit Peeler with Swivel Blade for Kitchen</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>525</v>
-      </c>
-      <c r="I21" t="n">
-        <v>229</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the ultimate kitchen companion with our stainless steel swivel blade vegetable peeler . This essential tool is engineered for effortless peeling of various fruits and vegetables, making your food preparation quicker and more enjoyable. Its smooth swivel blade glides along contours, ensuring thin, efficient removal of skins without wasting pulp. The comfortable handle provides a steady grip, enhancing control and safety during use, while the durable stainless steel construction promises long-lasting performance in any kitchen. Key features Sharp swivel blade follows uneven produce surfaces for controlled, efficient peeling. Durable stainless steel construction ensures reliable everyday use and rust resistance. Comfortable cylindrical handle offers a steady, non-slip grip during foo&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/24591-1.jpg</t>
-        </is>
-      </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/24591-2.jpg</t>
-        </is>
-      </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/24591-3.jpg</t>
-        </is>
-      </c>
-      <c r="Z21" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/24591-4.jpg</t>
-        </is>
-      </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/24591-5.jpg</t>
-        </is>
-      </c>
-      <c r="AB21" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/24591-6.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="51" customHeight="1">
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>11035_apex_ss_chimta_1pc</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Durable Stainless Steel Chimta for Safe Kitchen Use</t>
-        </is>
-      </c>
-      <c r="H22" t="n">
-        <v>525</v>
-      </c>
-      <c r="I22" t="n">
-        <v>269</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the essential kitchen tool for safe and effortless food handling. This premium stainless steel chimta, crafted for durability and performance, ensures you can manage hot items with confidence and ease. Perfect for a variety of cooking tasks, it&amp;#x27;s designed to be a reliable addition to any home or commercial kitchen. Ensures secure handling of hot food, providing a strong, reliable grip for flipping, turning, and serving with confidence and ease. Crafted from high-quality stainless steel, offering exceptional durability, rust resistance, and long-lasting performance for daily kitchen tasks. Designed with heat-resistant construction, allowing safe and comfortable use when cooking on gas stoves, tandoors, or induction cooktops. Simplifies your cooking, ideal for effortlessly managing&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Chimta-WOSKU-01.jpg</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/477S.Schimta.jpg</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Chimta-02.jpg</t>
-        </is>
-      </c>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/11035_apex_ss_chimta_1pc.jpg</t>
-        </is>
-      </c>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Chimta-04.jpg</t>
-        </is>
-      </c>
-      <c r="AB22" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Chimta-size.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="51" customHeight="1">
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>12133_pots_n_pans_protectors_pad_3pc</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Felt Pots and Pans Protectors – Set of 3 Sizes | Bake &amp; Dwell</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>569</v>
-      </c>
-      <c r="I23" t="n">
-        <v>219</v>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Kitchen &amp; Dining</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Felt pots and pans protectors are essential kitchen accessories that prevent scratches and damage to your cookware and countertops. This set of 3 protectors, available in large (38cm), medium (35cm), and small (26cm), ensures versatile use across all your pots, pans, plates, and bowls. Made from eco-friendly polyester felt, these protectors absorb impact and prevent stacking damage while adding a layer of heat protection. Key features Prevents scratches and chips between cookware pieces during storage or transport. Set includes three sizes: large, medium, and small for versatile kitchen use. Made from durable, eco-friendly polyester felt with a non-slip texture. Protects countertops from heat damage and wear during cooking and storage. Washable and reusable for long-lasting protection and&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_25269f02-055a-4659-a291-500d76d2a632.jpg</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/ec19082a-e5f4-4e4c-b86b-c65ae1a03429.jpg</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_0f6aa29e-7d42-498c-bdea-1a4bed11a7b1.jpg</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_a24a3d9f-48ed-4e64-a242-183097085924.jpg</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/08_1b5c7773-d8de-4ed5-8534-4bfd25e3895b.jpg</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_918aca57-ed07-4823-90fc-f7beeab4b5ae.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="51" customHeight="1">
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>18209_tranparent_adhesive_hook_6pc</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Transparent Adhesive Hooks (6 Pcs) – Strong &amp; Reusable | GlimmerHome</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>595</v>
-      </c>
-      <c r="I24" t="n">
-        <v>229</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Transform your home organisation with our versatile 6-piece transparent adhesive hook set . These strong, damage-free wall hooks are perfect for decluttering kitchens, bathrooms, and living spaces without drilling or leaving residue. Enjoy a clean, organised environment with GlimmerHome&amp;#x27;s premium adhesive solution. Key features Damage-Free Adhesion: Each transparent adhesive hook features a separate backing strip that adheres firmly to flat surfaces like tiles, glass, metal, and painted walls, yet removes cleanly without leaving marks or damage. High Load Capacity: Designed for durability, these robust wall hooks can hold up to 3 kg, making them ideal for hanging towels, kitchen utensils, coats, bags, and more. Versatile &amp;amp; Multi-Purpose: Use these strong wall hooks in your kitchen for ladl&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/18209_6797fc84-afc2-466b-95f8-85630df2c85e.png</t>
-        </is>
-      </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04f0556f-6f62-4753-b7e7-1c93ed9374c3.jpg</t>
-        </is>
-      </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_548f39c8-7fd2-438e-bb25-36c27165b698.jpg</t>
-        </is>
-      </c>
-      <c r="Z24" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_5f77b3bb-bd98-4a6f-ac78-c644b98e92a7.jpg</t>
-        </is>
-      </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/017_9155afd4-927a-4888-8b1c-35ed4bca6832.jpg</t>
-        </is>
-      </c>
-      <c r="AB24" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_f7bd0aa4-9449-4a5b-831b-1f6ee70f0368.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="51" customHeight="1">
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>whl175_94381_wg_1103_mix</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>LED Study Lamp with 3 Brightness Modes, Touch Control &amp; Flexible Neck (Color may vary)</t>
-        </is>
-      </c>
-      <c r="H25" t="n">
-        <v>509</v>
-      </c>
-      <c r="I25" t="n">
-        <v>319</v>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Brighten your workspace or study area with our versatile flexible neck LED desk lamp. This modern lamp features three adjustable brightness modes (Low, Medium, High) to suit any task, easily controlled with a sensitive touch button on its base. The flexible silicone gooseneck allows for effortless positioning, directing light exactly where you need it, making it perfect for reading, studying, working, or as a bedside light. Its compact design and non-slip base ensure stability on any surface, from study tables to office desks and kids&amp;#x27; rooms. Conveniently USB powered, this flexible neck LED desk lamp is an essential for efficient and comfortable lighting. Key features 3 Brightness Levels: Easily switch between Low, Medium, and High light modes for optimal visibility. Touch Control: Simple&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/6ObziZgHB0.jpg</t>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4WYl48GuEt.jpg</t>
-        </is>
-      </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/hh7UyUhSXR.jpg</t>
-        </is>
-      </c>
-      <c r="Z25" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/G3T8shx0jb.jpg</t>
-        </is>
-      </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Kf9qrNrAh3.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="51" customHeight="1">
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>whl282_13405_cartoon_led_desk_lamp_1pc</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Kids LED Desk Lamp – Cute Cartoon Eye-Protection | Deodap</t>
-        </is>
-      </c>
-      <c r="H26" t="n">
-        <v>510</v>
-      </c>
-      <c r="I26" t="n">
-        <v>349</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Brighten up your child&amp;#x27;s study space or bedside with our adorable Kids LED Desk Lamp from Deodap. Designed with a charming cartoon character base, this flexible and portable lamp provides soft, eye-friendly illumination, making it perfect for reading, homework, or a comforting night light. Its advanced luminous technology ensures there&amp;#x27;s no harsh glare, safeguarding your little one&amp;#x27;s eyes during long study sessions or quiet bedtime stories. Give them the gift of comfortable and fun lighting with this versatile LED lamp. This delightful Kids LED Desk Lamp combines playful aesthetics with practical functionality. Whether placed on a study table, bedside cabinet, or carried around for creative play, its lightweight and flexible design adapts to various needs. The USB rechargeable feature adds&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/13405_cartoon_led_desk_lamp_1pc.jpg</t>
-        </is>
-      </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/d8dad9aa-d991-4606-a71f-561e6256a024.jpg</t>
-        </is>
-      </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_59ead39c-d786-4226-8b68-7979a4ba3661.jpg</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_1576a615-9884-4df5-bc62-8acad894791d.jpg</t>
-        </is>
-      </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_bde756db-bd43-4bea-9032-87fe6dcf789f.jpg</t>
-        </is>
-      </c>
-      <c r="AB26" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_333169df-d3f6-4529-9cb7-63be3d9e1164.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="51" customHeight="1">
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>23627_cute_panda_night_lamp_1pc</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Cute Panda Showpiece Night Light for Kids Room Table &amp; Home Decor</t>
-        </is>
-      </c>
-      <c r="H27" t="n">
-        <v>439</v>
-      </c>
-      <c r="I27" t="n">
-        <v>249</v>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Add a cute and playful touch to your space with this adorable panda showpiece . Featuring a cheerful panda expression, raised paws, and attractive detailing, this compact showpiece is ideal for decorating kids&amp;#x27; rooms, study tables, desks, shelves, and bedside tables. Its charming design also makes it a lovely gifting option for children, friends, and panda lovers. Key Features Cute Panda Design: Adorable facial expression with attractive black, white, pink, and green detailing. Compact Decorative Showpiece: Easy to place on tables, desks, shelves, and cabinets. Kids Room Decor: Adds a fun and cheerful touch to children&amp;#x27;s rooms and study areas. Multipurpose Decoration: Suitable for home, bedroom, study table, office desk, and display shelf. Cute Gift Option: Ideal for birthdays, return gift&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/GFCe3rlgHp.jpg</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/ucrJjgY1AW.jpg</t>
-        </is>
-      </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/nIy5BvRK2Q.jpg</t>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/VHw3tFUnjw.jpg</t>
-        </is>
-      </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/dsVOdM1a8j.jpg</t>
-        </is>
-      </c>
-      <c r="AB27" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4A7fcmAQ14.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="51" customHeight="1">
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>4654_6pc_flexible_wall_hook</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Wall Hook Rail – Heavy Duty 6-Pin Transparent Golden | GlimmerHome</t>
-        </is>
-      </c>
-      <c r="H28" t="n">
-        <v>489</v>
-      </c>
-      <c r="I28" t="n">
-        <v>219</v>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Upgrade your home organisation with the Transparent 6-hook adhesive wall rail , designed to bring both style and exceptional utility to any space. Crafted for Indian homes, this heavy-duty 6-pin organiser helps declutter your living areas, offering a smart solution for hanging essentials. Its unique transparent and golden finish adds a touch of modern sophistication, making it more than just a functional item – it&amp;#x27;s a decor enhancer. Say goodbye to cluttered countertops and misplaced items. This versatile Transparent 6-hook adhesive wall rail is perfect for entryways, bathrooms, bedrooms, and kitchens, providing convenient access to coats, keys, towels, and accessories. Experience the blend of durability and design that GlimmerHome brings to your daily life, simplifying your home organisat&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Transparent-6-Wall-Hook-Using-1500x1500.png</t>
-        </is>
-      </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4654_7e0d08fc-1d7b-4546-a853-669e04f99943.jpg</t>
-        </is>
-      </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/07_6c983aa7-83e3-4e60-9f3d-8e9a2a8457fa.jpg</t>
-        </is>
-      </c>
-      <c r="Z28" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/06_c0cb4c30-a185-49c9-bbed-6d75bc1569da.jpg</t>
-        </is>
-      </c>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/08_c889bba5-02b7-4236-b77b-f8b024f2277e.jpg</t>
-        </is>
-      </c>
-      <c r="AB28" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_0424d040-e5e1-4363-8a95-e79fc589719f.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="51" customHeight="1">
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>17597_decor_round_mehndi_name_plate_1pc</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Mehndi Ceremony Wall Hanging – Lightweight Round Decorative Sign</t>
-        </is>
-      </c>
-      <c r="H29" t="n">
-        <v>485</v>
-      </c>
-      <c r="I29" t="n">
-        <v>259</v>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Enhance your wedding with this Mehndi ceremony wall hanging, designed to bring a traditional and festive charm to your mehndi, haldi, sangeet, or pre-wedding décor. This lightweight round decorative sign features the Hindi “मेहंदी” cut-out lettering, making it an eye-catching backdrop element perfect for photo booths, stage styling, or entrance decorations. Key features Bold round wall sign with Hindi “मेहंदी” lettering for instant cultural theme décor Lightweight and reusable design for easy installation and storage Pre-drilled holes for quick hanging using hooks, nails, strings, or double-sided tape Smooth, wipe-clean surface that resists creasing unlike paper decorations Complements floral curtains, fairy lights, drapes, and balloons for elegant styling Travel-friendly for versatile use&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W29" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Mehndi-wall-Decoration-01.jpg</t>
-        </is>
-      </c>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/102517597-99Pc-Mahendi-Av-Sv.jpg</t>
-        </is>
-      </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Mehndi-wall-Decoration-06.jpg</t>
-        </is>
-      </c>
-      <c r="Z29" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Mehndi-wall-Decoration-02.jpg</t>
-        </is>
-      </c>
-      <c r="AA29" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Mehndi-wall-Decoration-05.jpg</t>
-        </is>
-      </c>
-      <c r="AB29" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Mehndi-wall-Decoration-03.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="51" customHeight="1">
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>whl175_77886_1723_3</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Lord Ganesha Hanging Suncatcher Wall Decor for Home, Balcony &amp; Car</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
-        <v>539</v>
-      </c>
-      <c r="I30" t="n">
-        <v>399</v>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Enhance your home with the divine presence of this Lord Ganesha glass hanging decor. Featuring a vibrant Ganesha illustration, this decorative piece symbolizes wisdom, prosperity, and positive energy for any space. Key features Divine Lord Ganesha Design: Symbolizes wisdom, prosperity, protection, and positive energy for your home. Premium Hanging Cord: Durable natural jute rope with decorative beads adds a stylish finish. Multi-Purpose Decoration: Suitable for living room, pooja room, balcony, window, yoga room, meditation space, office, and car. Bright And Attractive Artwork: Vibrant colors add elegance and spiritual charm to any decor. Easy to Hang: Lightweight and ready to hang on hooks, walls, windows, or doors. Ideal Gift: Perfect for Diwali, Ganesh Chaturthi, housewarming, weddings,&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/BEWKLC04mY.png</t>
-        </is>
-      </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/wJ201azNKz.png</t>
-        </is>
-      </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/wCD72wwif2.png</t>
-        </is>
-      </c>
-      <c r="Z30" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4DFiLQ8IUO.png</t>
-        </is>
-      </c>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/FU2YHsgGEM.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="51" customHeight="1">
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>whl294_79825_17423_2_mix</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>DIY Tulip Mirror Lamp Kit - Colorful LED Night Light Decor</t>
-        </is>
-      </c>
-      <c r="H31" t="n">
-        <v>485</v>
-      </c>
-      <c r="I31" t="n">
-        <v>349</v>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Unleash your creativity and brighten any space with the captivating DIY Tulip Mirror Lamp Kit. This unique craft project transforms into a beautiful decorative light, featuring vibrant tulip flowers encased within reflective mirror panels. Enjoy the enchanting glow when lit, or the sleek mirror aesthetic when off, adding a touch of elegance to your home décor. Engage in a delightful DIY craft experience by assembling your own enchanting floral lamp, perfect for creative minds and décor enthusiasts. Experience a stunning visual transformation as colorful LED tulips illuminate when switched on, reflecting beautifully in the mirror panels. Adorn your space with a charming mix of pink, blue, yellow, and purple tulip-style flowers, creating an attractive and vibrant decorative display. Immerse&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/u8drG5EhUt.jpg</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/CATOkciJbJ.jpg</t>
-        </is>
-      </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Epb3Ml6Jfb.jpg</t>
-        </is>
-      </c>
-      <c r="Z31" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/63AYFzw0Qy.jpg</t>
-        </is>
-      </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/5uHg5DzVvg.jpg</t>
-        </is>
-      </c>
-      <c r="AB31" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/DGnfKB1TaP.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="51" customHeight="1">
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>21058_cube_tulip_flower_night_lamp_set</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Tulip Flower LED Cube Night Lamp – Warm Ambient Decorative Light</t>
-        </is>
-      </c>
-      <c r="H32" t="n">
-        <v>499</v>
-      </c>
-      <c r="I32" t="n">
-        <v>349</v>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Elevate your home atmosphere with the Tulip Flower LED Cube Night Lamp, a perfect blend of elegant design and soothing illumination. This decorative tulip flower LED cube lamp casts a warm ambient glow that enhances any room&amp;#x27;s mood and style. Key features Transparent cube design featuring a glowing tulip flower pattern Soft, warm LED light ideal for calming and ambient illumination Perfect for bedside, tabletop decor, and mood lighting Compact and lightweight for versatile placement on shelves and corners Enhances your home decor with a stylish floral accent Suitable for festive decoration and gifting on special occasions FAQ Q1: What is a Tulip Flower LED Cube Night Lamp? A: It&amp;#x27;s a decorative LED cube lamp with illuminated tulip flower patterns providing warm ambient lighting for home dec&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/21058_cube_tulip_flower_night_lamp_set_showcase_9d041eca-ef47-441b-b6c4-254c25047868.png</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/01_LED-Mirror.jpg</t>
-        </is>
-      </c>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_LED-Mirror.jpg</t>
-        </is>
-      </c>
-      <c r="Z32" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/06_LED-Mirror.jpg</t>
-        </is>
-      </c>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_LED-Mirror.jpg</t>
-        </is>
-      </c>
-      <c r="AB32" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_LED-Mirror.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="51" customHeight="1">
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>whl175_77890_634_1</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Cute Panda LED Night Lamp for Kids Room Bedroom &amp; Table Decor</t>
-        </is>
-      </c>
-      <c r="H33" t="n">
-        <v>489</v>
-      </c>
-      <c r="I33" t="n">
-        <v>249</v>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Brighten up any child&amp;#x27;s space with this adorable Panda LED Night Lamp. Featuring a charming panda character wearing a playful green leaf hat, this lamp emits a soft, warm glow, creating a comforting and cosy atmosphere in kids&amp;#x27; rooms and bedrooms. Its compact design makes it a versatile decorative piece for bedside tables, study desks, shelves, or nightstands, adding a touch of whimsy and warmth to any decor. Key features Adorable Panda Design: Features a cute panda with a unique green leaf-style top. Soft LED Illumination: Provides a gentle, warm light perfect for a relaxing nighttime ambience. Ideal for Kids&amp;#x27; Rooms: Attractive and safe lighting option suitable for children&amp;#x27;s bedrooms. Compact Tabletop Size: Easily fits on bedside tables, desks, and shelves. Decorative Accent: Adds a chee&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/FKUenUuiTR.jpg</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/qrWMMj8Ix0.jpg</t>
-        </is>
-      </c>
-      <c r="Y33" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4aHVA4gast.jpg</t>
-        </is>
-      </c>
-      <c r="Z33" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/ey2n5tAG2O.jpg</t>
-        </is>
-      </c>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/yeIr4pK2bc.jpg</t>
-        </is>
-      </c>
-      <c r="AB33" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/qLsafc32Mr.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="51" customHeight="1">
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>21255_cute_mini_panda_night_light_lamp</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Cute Mini Panda Night Light – Soft LED Bedside Lamp for Kids</t>
-        </is>
-      </c>
-      <c r="H34" t="n">
-        <v>440</v>
-      </c>
-      <c r="I34" t="n">
-        <v>289</v>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Home Decor</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The cute mini panda night light is designed to provide a gentle, calming glow that helps children feel safe and cozy at night. Perfect for bedrooms, nurseries, and study desks, this adorable panda lamp combines charming decor with functional lighting, creating a relaxing atmosphere for restful sleep. Its compact size makes it an ideal bedside companion, offering a soft, soothing light that does not disturb sleep patterns. Key features Cute panda design enhances room decor and adds a playful touch Soft LED light creates a calming, cozy ambiance Ideal as a night lamp for peaceful sleep and bedtime routines Compact and lightweight, perfect for small spaces and portable use Energy-efficient lighting saves power while illuminating effectively Child-safe and durable design ensures peace of mind&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Lightpanda-WOSKU-01.jpg</t>
-        </is>
-      </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/21255.jpg</t>
-        </is>
-      </c>
-      <c r="Y34" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Lightpanda-03.jpg</t>
-        </is>
-      </c>
-      <c r="Z34" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Lightpanda-06.jpg</t>
-        </is>
-      </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Lightpanda-04.jpg</t>
-        </is>
-      </c>
-      <c r="AB34" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Lightpanda-07.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="51" customHeight="1">
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>4785_selfie_ring_light</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Selfie Ring Light – Portable LED for Flawless Photos &amp; Videos | Gambit</t>
-        </is>
-      </c>
-      <c r="H35" t="n">
-        <v>470</v>
-      </c>
-      <c r="I35" t="n">
-        <v>299</v>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Transform your photos and videos with the ultimate Selfie Ring Light from Gambit, designed to provide professional-grade illumination wherever you go. Say goodbye to dull, poorly lit shots and hello to vibrant, perfectly exposed content. This portable ring light is an essential tool for creators, beauty enthusiasts, and anyone looking to enhance their digital presence with brilliant lighting. Whether you&amp;#x27;re taking a quick selfie, recording a detailed makeup tutorial, or engaging in video calls, this LED ring light ensures you always look your best. Its lightweight and compact design makes it incredibly easy to carry, fitting seamlessly into your bag or purse. Experience the difference a dedicated light source makes, providing even, soft illumination that eliminates harsh shadows and brings&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W35" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/01_9517595e-8d48-451f-91b7-e252bf2d5beb.jpg</t>
-        </is>
-      </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/F3KmSjCQqupnir8zXY8mlr2ezuDOTMSE6vAlE6DE.jpg</t>
-        </is>
-      </c>
-      <c r="Y35" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/10_0d64f988-9475-46ff-b89d-9a7f34df7618.jpg</t>
-        </is>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/2092621090.png</t>
-        </is>
-      </c>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/2092621089.png</t>
-        </is>
-      </c>
-      <c r="AB35" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/08_c074b9b2-7a8c-42fb-bac4-2024d4b136cb.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="51" customHeight="1">
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>whl282_4810_portable_desk_fan_big</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Portable Desk Fan – Quiet 3-Speed USB Power for Home &amp; Office | VoltDesk</t>
-        </is>
-      </c>
-      <c r="H36" t="n">
-        <v>455</v>
-      </c>
-      <c r="I36" t="n">
-        <v>299</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Stay cool and comfortable anywhere with the **Mint green portable USB desk fan** from VoltDesk. Designed for ultimate convenience and efficiency, this compact yet powerful fan is your perfect companion for home, office, study, or travel. Experience a refreshing breeze without distracting noise, thanks to its advanced brushless motor and energy-saving USB power compatibility. Whether you&amp;#x27;re working, relaxing, or on the go, this Mint green portable USB desk fan ensures a steady, quiet airflow to keep you comfortable through the Indian summers. This versatile mini table fan is engineered for modern lifestyles, offering not just portability but also robust performance. Its thoughtful design includes a protective fence cover for enhanced safety, making it suitable for use around children and pe&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W36" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4810_portable_desk_fan_big.jpg</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4810_1.jpg</t>
-        </is>
-      </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4810.jpg</t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4810_2.jpg</t>
-        </is>
-      </c>
-      <c r="AA36" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4810_3.jpg</t>
-        </is>
-      </c>
-      <c r="AB36" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/4810_5.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="51" customHeight="1">
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>22669_mini_usb_fan_1pc</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Portable USB Mini Fan – Compact &amp; Adjustable for Personal Cooling</t>
-        </is>
-      </c>
-      <c r="H37" t="n">
-        <v>475</v>
-      </c>
-      <c r="I37" t="n">
-        <v>219</v>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The Portable USB Mini Flexible Fan is your ideal solution for personal cooling on the go. With its bendable neck, you can direct airflow precisely where needed, making it perfect for workspaces, travel, and outdoor activities. Its compact design ensures portability without sacrificing performance, while being USB-powered means it’s compatible with laptops, power banks, and USB adapters for convenience anywhere you need a quick cool-down. Key features Flexible bendable neck for customized airflow direction USB powered for compatibility with laptops, power banks, and wall adapters Small, lightweight, and portable design ideal for travel and outdoor use Quiet operation suitable for office, study, or personal spaces Energy-efficient with durable construction for long-lasting use Materials &amp;amp; ca&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W37" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/PoweredMiniFan-WOSKU-01.jpg</t>
-        </is>
-      </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/sku_4175b6cb-c6c1-4235-bf70-6662635ced44.jpg</t>
-        </is>
-      </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/PoweredMiniFan-6.jpg</t>
-        </is>
-      </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/PoweredMiniFan-04.jpg</t>
-        </is>
-      </c>
-      <c r="AA37" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/PoweredMiniFan-05.jpg</t>
-        </is>
-      </c>
-      <c r="AB37" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/PoweredMiniFan-size.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="51" customHeight="1">
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>6183_mini_usb_fan</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Mini USB Fan Portable Mobile Phone Plug In Cooling Fan Soft Blades</t>
-        </is>
-      </c>
-      <c r="H38" t="n">
-        <v>599</v>
-      </c>
-      <c r="I38" t="n">
-        <v>229</v>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Stay cool anywhere with this green portable USB-C phone fan. Designed for convenience, this mini fan plugs directly into your smartphone, offering instant personal cooling. Its soft, flexible blades ensure safety, making it perfect for travel, outdoor activities, or simply beating the summer heat. Key features Plugs directly into your mobile phone for instant personal cooling on the go Soft flexible blades are safe to touch and will not hurt fingers during use Compact and lightweight design fits easily in pockets, bags, and travel kits No batteries required as it draws power directly from your smartphone via USB-C Powerful airflow provides refreshing cooling during hot summer days Simple plug and play operation with no setup or charging needed Ideal for travel, commuting, outdoor events, a&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W38" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniUSBFan-01.jpg</t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/sku_7568eccf-ac04-4a0b-a5ac-ed6145d5cecd.jpg</t>
-        </is>
-      </c>
-      <c r="Y38" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniUSBFan-05.jpg</t>
-        </is>
-      </c>
-      <c r="Z38" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniUSBFan-06.jpg</t>
-        </is>
-      </c>
-      <c r="AA38" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniUSBFan-04.jpg</t>
-        </is>
-      </c>
-      <c r="AB38" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniUSBFan-size.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="51" customHeight="1">
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>22877_5_mode_mini_led_keychain_flashligh</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>5 Mode Mini COB LED Keychain Flashlight with Carabiner Clip</t>
-        </is>
-      </c>
-      <c r="H39" t="n">
-        <v>539</v>
-      </c>
-      <c r="I39" t="n">
-        <v>329</v>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the versatility of the 5 Mode Mini COB LED Keychain Flashlight, your perfect companion for illumination on the go. This compact and powerful device, featuring a vibrant red and black design, ensures you always have light when you need it most. Ideal for everyday carry, it easily attaches to your keys or bag, providing reliable lighting for various situations. Key features Five lighting modes: high, low, strobe, SOS, and spotlight for adaptable use. Powerful COB LED panel offers bright, wide-area flood lighting. Secondary spotlight torch delivers a focused beam for longer distances. Built-in carabiner clip allows easy attachment to keys, bags, or belts. Ultra-compact, pocket-sized, and lightweight for effortless portability. Durable ABS plastic construction withstands daily use and&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W39" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniPortableFlashlightKeychain-01.jpg</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/sku_8c5297b5-e3ce-4c22-8bcd-73584449baa9.jpg</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniPortableFlashlightKeychain-02.jpg</t>
-        </is>
-      </c>
-      <c r="Z39" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniPortableFlashlightKeychain-04.jpg</t>
-        </is>
-      </c>
-      <c r="AA39" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniPortableFlashlightKeychain-03.jpg</t>
-        </is>
-      </c>
-      <c r="AB39" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/MiniPortableFlashlightKeychain-size.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="51" customHeight="1">
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>13978_mini_light_up_torch</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Mini LED Torch – Compact, Portable &amp; Bright Light</t>
-        </is>
-      </c>
-      <c r="H40" t="n">
-        <v>629</v>
-      </c>
-      <c r="I40" t="n">
-        <v>229</v>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the convenience of our Blue mini disco ball light wand, a compact and portable solution for reliable lighting and entertainment. This mini disco ball light wand is ideal for parties, events, or simply adding a fun ambiance to any room, providing bright, colourful illumination where you need it most. Lightweight and durable, it&amp;#x27;s designed for easy carrying and delivers efficient, long-lasting light with a captivating disco ball effect. Key features Compact size (10 cm length) for ultimate portability and easy handling Bright LED lights with a captivating mini disco ball effect Lightweight design, weighing just 35 grams, for effortless carrying Durable construction suitable for various indoor and outdoor settings Simple on/off switch for quick and easy operation Perfect for parties,&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W40" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/13978.png</t>
-        </is>
-      </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/3a5b73d1-bf19-4022-8c2a-db440ea0a35d.jpg</t>
-        </is>
-      </c>
-      <c r="Y40" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_5f2c06c6-3367-44a6-be67-2e2f8fdcb255.jpg</t>
-        </is>
-      </c>
-      <c r="Z40" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_27406132-5058-4c6f-b0d0-3393c17bc9b7.jpg</t>
-        </is>
-      </c>
-      <c r="AA40" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_5742c6ca-7314-4e59-a2fa-54a570fd9d09.jpg</t>
-        </is>
-      </c>
-      <c r="AB40" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_b71c037b-f863-4f69-ab9b-53e09f4b7102.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="51" customHeight="1">
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>6251_5in1_multifunction_brush</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Computer Cleaning Kit – 5-in-1 Multi-Function PC &amp; Keyboard | Dustiva</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>479</v>
-      </c>
-      <c r="I41" t="n">
-        <v>249</v>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Keep your digital world spotless with the ultimate Computer Cleaning Kit from Dustiva. This 5-in-1 multi-function tool is meticulously designed to tackle every speck of dust and grime from your precious electronics, ensuring they look new and perform optimally. Perfect for gamers, professionals, and everyday users in India, this kit is your go-to solution for comprehensive device maintenance, enhancing longevity and performance for your PC, keyboard, and earbuds. Key features 5-in-1 Comprehensive Cleaning: Includes a metal pen tip for stubborn grime, a high-density brush, a soft flocking sponge for delicate surfaces, a robust keyboard brush, and an easy-to-use keycap puller. Precision Earbuds Cleaning: The delicate flocking sponge and metal pen tip are perfect for cleaning wireless earbud&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W41" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/3image_2793e13d-4fea-4a76-b3d9-af8a42520c96.jpg</t>
-        </is>
-      </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/1image_c52a168c-ae61-4870-8128-c0d76696cef6_1.jpg</t>
-        </is>
-      </c>
-      <c r="Y41" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/2image_be686450-a4f9-4053-aad1-666afcaa5443.jpg</t>
-        </is>
-      </c>
-      <c r="Z41" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/7image_34fbcf4e-da9d-4bbb-a106-90222c272fa0.jpg</t>
-        </is>
-      </c>
-      <c r="AA41" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/4image_cc4a377e-c606-41f2-bfb3-251d61415521.jpg</t>
-        </is>
-      </c>
-      <c r="AB41" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/5image_7e463727-3a9c-4118-8718-49609b03d19a.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="51" customHeight="1">
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>6124_4pc_multi_p_mob_stand</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Wall Mounted Phone Holder – Multi-functional Organizer | Organivo</t>
-        </is>
-      </c>
-      <c r="H42" t="n">
-        <v>515</v>
-      </c>
-      <c r="I42" t="n">
-        <v>239</v>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Transform your living space and keep essentials neatly organised with our innovative Wall Mounted Phone Holder . This multi-functional organiser is designed to declutter your bedside, desk, or kitchen, providing a dedicated spot for your smartphone and remote controls. Say goodbye to misplaced remotes and tangled charging cables; this sleek solution from Organivo ensures everything is always within reach and perfectly tidy. Key features Dual Functionality: Serves as both a secure wall mounted phone holder and a convenient remote control organizer. Integrated Charging Port: Thoughtfully designed with a bottom opening, allowing you to charge your phone effortlessly while it rests in the holder. Easy, Damage-Free Installation: Features strong adhesive backing for quick and simple mounting on&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U42" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W42" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/3b9a0d7f-a23d-4029-b99f-358519825831.jpg</t>
-        </is>
-      </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/01_ad372f27-1965-4137-b508-425ee0c62640.jpg</t>
-        </is>
-      </c>
-      <c r="Y42" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/01_120dc563-a380-41e0-a7ac-df7cd114dd49.jpg</t>
-        </is>
-      </c>
-      <c r="Z42" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/07_eebea5d0-1b3a-4f9d-a82e-b8e5ac760d57.jpg</t>
-        </is>
-      </c>
-      <c r="AA42" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/04_1667da0d-6ab3-4afb-8014-6ef3b3cf7eb7.jpg</t>
-        </is>
-      </c>
-      <c r="AB42" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/products/08_a3feea56-c6d4-4edb-8158-53709169177f.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="51" customHeight="1">
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>23927_4_port_usb_to_usb</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>USB to Four Port USB Hub Multi Interface Adapter for Laptop and Computer</t>
-        </is>
-      </c>
-      <c r="H43" t="n">
-        <v>475</v>
-      </c>
-      <c r="I43" t="n">
-        <v>289</v>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Expand your connectivity with this versatile Silver 4-port USB hub adapter . Designed for both laptops and desktop computers, this compact device effortlessly transforms a single USB port into four, allowing you to connect multiple peripherals simultaneously. Ideal for decluttering your workspace or enhancing your travel accessory kit, this hub ensures seamless data transfer and device connectivity for everyday use. Key features Multi-interface USB hub design for expanded connectivity Standard USB input connector for universal compatibility Connects multiple USB accessories with ease Compact and lightweight body for portability Flexible attached connecting cable for convenient placement Simple plug-and-use design requires no drivers Suitable for both desk and on-the-go use Sleek silver and&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W43" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23927-USB-Splitter-multiport-Adapter-1.jpg</t>
-        </is>
-      </c>
-      <c r="X43" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23927-sku.jpg</t>
-        </is>
-      </c>
-      <c r="Y43" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23927-USB-Splitter-multiport-Adapter-2.jpg</t>
-        </is>
-      </c>
-      <c r="Z43" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23927-USB-Splitter-multiport-Adapter-3.jpg</t>
-        </is>
-      </c>
-      <c r="AA43" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23927-USB-Splitter-multiport-Adapter-7.jpg</t>
-        </is>
-      </c>
-      <c r="AB43" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23927-USB-Splitter-multiport-Adapter-6.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="51" customHeight="1">
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>23597_usb_rechargeable_led_flashlight</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>USB Rechargeable LED Flashlight for Travel with Lamp Mode</t>
-        </is>
-      </c>
-      <c r="H44" t="n">
-        <v>559</v>
-      </c>
-      <c r="I44" t="n">
-        <v>349</v>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;USB Rechargeable LED Flashlight for Travel with Soft Lamp Mode for Trips, Camping and Night Use (1 Pc) Description :- A phone torch drains the battery you need for maps and calls, which is the wrong trade on a trip. This flashlight does the lighting so the phone does not have to. The beam covers a dark path or a hotel corridor, and the soft lamp mode gives enough light to find something in a bag without waking the person next to you. USB charging means the same cable that charges your phone charges this, so there is nothing extra to pack. Key Features Saves the phone battery you need for maps and calls Beam covers a dark path, corridor or campsite Soft lamp mode for finding things in a bag without waking anyone Charges off the same USB cable as your phone No batteries to carry or buy on th&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W44" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/c23b24ee-e8ec-4f49-a6a3-7fd08ff805ca.jpg</t>
-        </is>
-      </c>
-      <c r="X44" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/d52ec2cc-e497-44d8-9c22-089d55f3fd44.jpg</t>
-        </is>
-      </c>
-      <c r="Y44" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23597-usb-rechargeable-led-flashlight-3.jpg</t>
-        </is>
-      </c>
-      <c r="Z44" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23597-usb-rechargeable-led-flashlight-4.jpg</t>
-        </is>
-      </c>
-      <c r="AA44" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23597-usb-rechargeable-led-flashlight-5.jpg</t>
-        </is>
-      </c>
-      <c r="AB44" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/23597-usb-rechargeable-led-flashlight-6.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="51" customHeight="1">
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>1637_usb_bike_light</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>USB Rechargeable Bicycle Headlight with Handlebar Mount for Night Riding</t>
-        </is>
-      </c>
-      <c r="H45" t="n">
-        <v>499</v>
-      </c>
-      <c r="I45" t="n">
-        <v>299</v>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Smart Gadgets</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Enhance your cycling safety with our USB rechargeable bicycle headlight , designed for superior visibility during night rides and low-light conditions. This reliable headlight ensures you can see the path ahead clearly and be seen by others, making your evening commutes and early morning adventures safer. Its compact design and easy handlebar mount make it a convenient and essential accessory for every cyclist. Key features Bright front beam provides excellent visibility in low-light conditions. USB rechargeable design eliminates the need for disposable batteries, offering an eco-friendly solution. Secure mounting bracket easily attaches to bicycle handlebars for stable positioning. Compact and lightweight body ensures it won&amp;#x27;t add unnecessary bulk to your bike. Simple control button allow&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U45" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W45" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/1637-01.jpg</t>
-        </is>
-      </c>
-      <c r="X45" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/1637-02.jpg</t>
-        </is>
-      </c>
-      <c r="Y45" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/1637-03.jpg</t>
-        </is>
-      </c>
-      <c r="Z45" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/1637-04.jpg</t>
-        </is>
-      </c>
-      <c r="AA45" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/1637-05.jpg</t>
-        </is>
-      </c>
-      <c r="AB45" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/1637-06.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="51" customHeight="1">
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>whl193_66653_dryfruit_box_open_square_de</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Royal Decorative Dry Fruit Box for Festive Serving &amp; Gifting</t>
-        </is>
-      </c>
-      <c r="H46" t="n">
-        <v>449</v>
-      </c>
-      <c r="I46" t="n">
-        <v>349</v>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Elevate your entertaining and gifting with the Royal Decorative Dry Fruit Box, a stunning piece designed to add elegance to any occasion. Perfect for showcasing an array of treats, from crunchy nuts to delightful sweets, this box combines traditional charm with practical functionality. Its exquisite design makes it a focal point on any table, embodying a sense of luxury and thoughtful presentation for both everyday use and special celebrations. Showcase Treats Elegantly: Designed for stylish serving and storage, this box beautifully displays nuts, dry fruits, sweets, and snacks, making every presentation special. Adds Royal Decorative Flair: Featuring a premium decorative design, it infuses a luxurious and traditional touch into your dining table and festive home decor instantly. Offers Ea&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W46" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/iK4vbVtSFD.jpg</t>
-        </is>
-      </c>
-      <c r="X46" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/oVYvpUeGUz.jpg</t>
-        </is>
-      </c>
-      <c r="Y46" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/VxXcStBWAR.jpg</t>
-        </is>
-      </c>
-      <c r="Z46" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/mQd4WElKJY.jpg</t>
-        </is>
-      </c>
-      <c r="AA46" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/YAiVLYzI9T.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="51" customHeight="1">
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>14409_gold_metal_medal_n_tricolor_ribbon</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Gold Medal Gift with Tricolor Ribbon for Achievers, Kids and Winners (1 Pc)</t>
-        </is>
-      </c>
-      <c r="H47" t="n">
-        <v>505</v>
-      </c>
-      <c r="I47" t="n">
-        <v>219</v>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Celebrate success and milestones with this elegant Gold Medal Gift. Featuring a shiny gold finish and a vibrant tricolor ribbon, this award medal is a perfect keepsake for achievers of all ages. Ideal for recognising academic excellence, sports victories, or simply celebrating personal achievements, it makes a memorable token of pride and appreciation. Key features Gift of Pride: Celebrate achievements big and small. Gold Finish: Shiny, premium look. Tricolor Ribbon: Comfortable to wear around the neck. For All Ages: Suitable for kids and adults. Keepsake Gift: A lasting memory of a special moment. Many Occasions: Results, birthdays, sports and competitions. Lightweight: Easy to wear and carry. Easy Care: Wipe with a soft cloth to keep it shining. Materials &amp;amp; care Material: Metal with Fabr&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W47" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_439c02be-7e1a-45ae-9e16-fd6413cd5580.jpg</t>
-        </is>
-      </c>
-      <c r="X47" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/14409.jpg</t>
-        </is>
-      </c>
-      <c r="Y47" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_d002869f-bad7-469c-8675-e6142dd728bc.jpg</t>
-        </is>
-      </c>
-      <c r="Z47" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_7de3e992-f6bf-4f9d-b0bb-4c4ac376125c.jpg</t>
-        </is>
-      </c>
-      <c r="AA47" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/07_800a7bc3-2477-4210-b220-6e490514726e.jpg</t>
-        </is>
-      </c>
-      <c r="AB47" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/06_c18f5d4c-5cec-4262-b366-1e49c92c7c1d.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="51" customHeight="1">
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>whl282_19630_krishna_flute_metal_keychai</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Krishna Flute Keychain – Durable Stainless Steel Spiritual Accessory</t>
-        </is>
-      </c>
-      <c r="H48" t="n">
-        <v>499</v>
-      </c>
-      <c r="I48" t="n">
-        <v>219</v>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Experience divine blessings with our Krishna flute keychain, crafted from premium stainless steel for durability and spiritual elegance. This keychain features the iconic image of Lord Krishna holding his mystical flute, symbolizing love, harmony, and devotion. Perfect for organizing car, bike, home, or office keys while keeping the positive energy of Krishna close. Key features Intricate Krishna flute design with precise laser-cut detailing High-quality stainless steel resistant to rust and wear Compact and lightweight for effortless everyday carry Strong metal ring securely holds multiple keys Polished finish adding a sleek and stylish look Ideal as a thoughtful gift for Janmashtami, Diwali, or other festivities Combines spiritual significance with practical utility Materials &amp;amp; care Made&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W48" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Krishna-keychain-02_166f48cb-9946-410b-83a4-4a6dd6a4f3be.jpg</t>
-        </is>
-      </c>
-      <c r="X48" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/c5751ef3-5e9c-4060-85ef-a406ca3f909a_63b6b3a7-3e12-49b2-8d0c-828e9063dce3.jpg</t>
-        </is>
-      </c>
-      <c r="Y48" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Krishna-keychain-01_dc3e06fe-f38d-4392-8ca0-bdb67e367317.jpg</t>
-        </is>
-      </c>
-      <c r="Z48" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Krishna-keychain-03_7878e90e-af45-49c2-b90b-a25ed15e63ca.jpg</t>
-        </is>
-      </c>
-      <c r="AA48" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Krishna-keychain-05_eabc8cf7-87cd-4d8b-aa87-8176020672c1.jpg</t>
-        </is>
-      </c>
-      <c r="AB48" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Krishna-keychain-06_016cbeeb-315b-4913-8cbb-c622007878d7.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="51" customHeight="1">
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>13177_adhesive_phone_card_holder_1pc</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Adhesive Card Phone Holder – Zipper Pocket Wallet | Mobiléon</t>
-        </is>
-      </c>
-      <c r="H49" t="n">
-        <v>469</v>
-      </c>
-      <c r="I49" t="n">
-        <v>349</v>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Streamline your everyday essentials with the innovative Adhesive Card Phone Holder from Mobiléon. This sleek and practical accessory easily attaches to the back of almost any smartphone or case, transforming it into a convenient mobile wallet. No more fumbling for your cards or cash – everything you need is securely right at your fingertips. Designed for the modern Indian user, this durable phone back wallet combines minimalist style with maximum functionality, making it perfect for anyone looking to lighten their load while staying organised on the go. Key features Secure Zipper Pocket: Safely store your essential cards, ID, and cash in a discreet, zippered compartment, offering enhanced security over open card slots. Strong Adhesive Backing: Equipped with a high-quality adhesive, this mo&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W49" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_d38833c7-983f-43a2-a1dd-741444d2a86c.jpg</t>
-        </is>
-      </c>
-      <c r="X49" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/2_7f3b98af-0baf-49f8-aa0b-eb72269a8e5a.jpg</t>
-        </is>
-      </c>
-      <c r="Y49" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/1_9c8c1859-bb0a-45b4-a1b7-804b63796155.jpg</t>
-        </is>
-      </c>
-      <c r="Z49" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/wallet-3.jpg</t>
-        </is>
-      </c>
-      <c r="AA49" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/wallet-7.jpg</t>
-        </is>
-      </c>
-      <c r="AB49" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/wallet-6.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="51" customHeight="1">
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>whl146_11521_apex_ss_cat_mug_250ml_cm_cp</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Apex Cat Mug – 250 ml Stainless Steel Insulated Kids' Mug</t>
-        </is>
-      </c>
-      <c r="H50" t="n">
-        <v>510</v>
-      </c>
-      <c r="I50" t="n">
-        <v>319</v>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;The Apex Cat Mug is a delightful insulated kids&amp;#x27; mug designed with a cute double-cat print to brighten up your child&amp;#x27;s beverage time. This 250 ml stainless steel insulated mug combines fun design with practical features like a leak-proof lid and durable plastic outer body, perfect for keeping drinks warm for longer while ensuring easy handling for little hands. Key features Adorable Cat Design: Features a colorful double-cat print adding a playful charm. Insulated Stainless Steel Inner: Keeps beverages at the ideal temperature longer, ideal for hot tea, milk, or soup. Durable Plastic Outer Body: Lightweight and break-resistant for safe daily use by kids. Leak-Proof Lid: Prevents spills ensuring mess-free transport in school bags or desks. Comfort Grip Handle: Ergonomically designed for sma&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/01_db6a104e-3139-4cde-985e-dd560fbbaed5.jpg</t>
-        </is>
-      </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/842a32ec-6bd0-4386-8711-1ba93fac9f16.jpg</t>
-        </is>
-      </c>
-      <c r="Y50" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_d07ebb01-1990-4b5e-9b72-25c0360be465.jpg</t>
-        </is>
-      </c>
-      <c r="Z50" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_62065805-7968-42b1-acdd-4b974ed1e1db.jpg</t>
-        </is>
-      </c>
-      <c r="AA50" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_9f1877c2-c4d5-4899-a616-291ee62b4bf8.jpg</t>
-        </is>
-      </c>
-      <c r="AB50" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/06_35f0202e-f4af-43be-ba5c-ae92c52950c2.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="51" customHeight="1">
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>whl282_12774_jewellery_gift_box_1pc</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Ring Gift Box – Premium Elegant Presentation with Velvet Cushion</t>
-        </is>
-      </c>
-      <c r="H51" t="n">
-        <v>439</v>
-      </c>
-      <c r="I51" t="n">
-        <v>249</v>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Ring gift box crafted to perfectly present and protect your precious jewelry with elegance. Its sturdy decorative exterior and soft velvet cushion make it ideal for gifting and storage of rings. Key features Elegant jewelry presentation box with decorative diamond-themed finish Soft velvet-lined interior cushion prevents scratches and holds rings securely Snap-style magnetic closure ensures the box remains firmly sealed Hard protective outer casing provides safe storage and durability Compact and lightweight design suitable for gifting and travel Striking contrast color enhances the overall luxurious appearance Perfect for proposals, engagements, anniversaries, and jewelry shop presentations Materials &amp;amp; care The box features a hard outer shell with a decorative finish and a soft velvet-lin&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Ringbox-WOSKU-01.jpg</t>
-        </is>
-      </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/19412774-128Pc-Ringbox-Av-Sv.jpg</t>
-        </is>
-      </c>
-      <c r="Y51" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Ringbox-05.jpg</t>
-        </is>
-      </c>
-      <c r="Z51" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Ringbox-06.jpg</t>
-        </is>
-      </c>
-      <c r="AA51" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Ringbox-04.jpg</t>
-        </is>
-      </c>
-      <c r="AB51" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/Ringbox-size.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="51" customHeight="1">
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>18916_plastic_flower_vase_1pc</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Plastic Flower Vase – Elegant Design for Home &amp; Gift</t>
-        </is>
-      </c>
-      <c r="H52" t="n">
-        <v>505</v>
-      </c>
-      <c r="I52" t="n">
-        <v>259</v>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the charm of the Plastic Flower Vase, crafted for elegant home decor and perfect as a thoughtful gift for family and friends. This plastic flower vase offers a sleek silhouette that enhances any room, bringing a fresh, decorative touch to your living room, office, or dining table. Key features Elegant and modern design with a smooth, textured finish for a refined look. Multipurpose vase suitable for fresh bouquets, artificial flowers, and silk greenery. Lightweight plastic construction ensures durability and easy handling. Ideal for home decor, office desk embellishment, bathroom, kitchen, or wedding centrepieces. An excellent gifting choice for birthdays, housewarmings, and special occasions. Compact size with dimensions: length 18 cm, width 7 cm, height 7 cm for versatile placem&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W52" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/01_91c87a05-2ddc-443d-aee5-5aaa0ccf7bb7.jpg</t>
-        </is>
-      </c>
-      <c r="X52" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/c7b8256b-ca06-449d-b7e2-4627ed71258c.jpg</t>
-        </is>
-      </c>
-      <c r="Y52" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/03_09ed9caa-6d17-4595-8fd7-d5da22d94de9.jpg</t>
-        </is>
-      </c>
-      <c r="Z52" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/04_7cda10fe-b23b-41b8-9646-9b6189b2cc87.jpg</t>
-        </is>
-      </c>
-      <c r="AA52" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/05_671810cd-b793-47bd-9932-d837eb7a22ca.jpg</t>
-        </is>
-      </c>
-      <c r="AB52" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/02_fe1fa176-7079-4eaf-ba0d-ae00d5d62249.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="51" customHeight="1">
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>whl282_22517_next_velvet_oud_attar_12ml</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Next Velvet Oud Attar – Long Lasting, Premium Fragrance Oil</t>
-        </is>
-      </c>
-      <c r="H53" t="n">
-        <v>510</v>
-      </c>
-      <c r="I53" t="n">
-        <v>369</v>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Discover the rich and luxurious scent of Next Velvet Oud Concentrated Attar Perfume 12 ML, designed for those who seek a deep, woody, and musky aroma that lasts for hours. This premium oud attar is ideal for individuals who appreciate traditional oriental fragrances with a modern twist. Crafted without alcohol, this unisex perfume offers a sophisticated,浓ent experience suitable for daily wear, special occasions, and religious gatherings. Its compact size makes it convenient for travel and on-the-go application, whether you prefer a roll-on or dab method. Key features Premium concentrated oud fragrance Long lasting and rich aroma Non alcoholic attar formula Suitable for men and women Elegant luxury bottle design Easy roll on or dab application 12 ML compact size Materials &amp;amp; care Maintain th&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U53" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W53" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/NextCareVelvetOudAttar-WOSKU-01.jpg</t>
-        </is>
-      </c>
-      <c r="X53" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/NextCareVelvetOudAttar-WSKU-01.jpg</t>
-        </is>
-      </c>
-      <c r="Y53" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/NextCareVelvetOudAttar-05.jpg</t>
-        </is>
-      </c>
-      <c r="Z53" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/NextCareVelvetOudAttar-04.jpg</t>
-        </is>
-      </c>
-      <c r="AA53" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/NextCareVelvetOudAttar-03.jpg</t>
-        </is>
-      </c>
-      <c r="AB53" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/NextCareVelvetOudAttar-size.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="51" customHeight="1">
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>8782_mini_jewelry_organizer_box</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Travel Jewellery Box – Portable PU Leather Organiser | LilyGleam</t>
-        </is>
-      </c>
-      <c r="H54" t="n">
-        <v>525</v>
-      </c>
-      <c r="I54" t="n">
-        <v>269</v>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Searching for the perfect travel jewellery box that combines style, functionality, and portability? Look no further than the LilyGleam Mini PU Leather Travel Jewellery Box. Designed for the modern Indian woman on the go, this elegant and compact organiser ensures your precious rings, necklaces, and earrings stay safe, secure, and tangle-free, whether you&amp;#x27;re heading to a weekend getaway or a business trip. Say goodbye to lost earrings and tangled chains with this essential accessory for every journey. Key features Compact &amp;amp; Portable Design: Perfectly palm-sized, this travel jewellery box easily fits into handbags, luggage, or carry-ons for convenient travel. Multi-Functional Storage: Thoughtfully designed compartments for rings, necklaces, earrings, studs, and even small makeup items like l&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U54" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W54" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/jewelry-box-1---05.jpg</t>
-        </is>
-      </c>
-      <c r="X54" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/8782.jpg</t>
-        </is>
-      </c>
-      <c r="Y54" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/jewelry-box-1---03.jpg</t>
-        </is>
-      </c>
-      <c r="Z54" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/jewelry-box-1---04.jpg</t>
-        </is>
-      </c>
-      <c r="AA54" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/jewelry-box-1---07.jpg</t>
-        </is>
-      </c>
-      <c r="AB54" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/jewelry-box-1---06.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="51" customHeight="1">
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>21611_golden_rose_n_box</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>Gold Plated Artificial Rose – Eternal Love Decor Gift</t>
-        </is>
-      </c>
-      <c r="H55" t="n">
-        <v>479</v>
-      </c>
-      <c r="I55" t="n">
-        <v>299</v>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;This gold plated artificial rose is a timeless symbol of eternal love and appreciation. Crafted with exquisite detail, this decorative golden rose perfectly expresses affection and serves as a lasting gift that never wethers, making it an ideal choice for special occasions or home decor. Key features Premium gold plating: The rose is coated with 24K gold foil, symbolising nobility and eternal love. Handcrafted artistry: Expert artisans precisely create each rose to capture the beauty of natural flowers. Elegant presentation: Comes in a beautiful purple premium box with a transparent front to showcase the rose without unboxing. Versatile decoration: Ideal for home, office decor, weddings, parties, or special occasions. Never fades or wilts: A lasting expression of love and best wishes that&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U55" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="W55" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/WhatsApp_Image_2026-08-27_at_18.57.15_20b57117-2e09-4f20-8eb5-393c691ed431.jpg</t>
-        </is>
-      </c>
-      <c r="X55" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/08_c7bb241f-04da-47c1-8994-392fb0134638.jpg</t>
-        </is>
-      </c>
-      <c r="Y55" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/whl175_67690_mn_033_go_3af2ed48-1c67-4301-b108-d55c01fa5eb1.jpg</t>
-        </is>
-      </c>
-      <c r="Z55" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/61ClF3UfoWL._SL1000_d63357b1-11b2-49f3-90f0-c7267d160838.jpg</t>
-        </is>
-      </c>
-      <c r="AA55" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/41nZL-LzlYL_0884f0a3-0f89-4e37-b20a-f67a189543c7.jpg</t>
-        </is>
-      </c>
-      <c r="AB55" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/51VptqPMk5L._SL1500_4de1596f-93c1-4a3f-b0d1-bf4af8467a34.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="51" customHeight="1">
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>22311_paper_long_rectangle_empty_gift_bo</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Long Rectangular Paper Empty Gift Box with Bow for Jewellery and Gifting</t>
-        </is>
-      </c>
-      <c r="H56" t="n">
-        <v>509</v>
-      </c>
-      <c r="I56" t="n">
-        <v>219</v>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Gifts &amp; Hampers</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Present your thoughtful gifts elegantly with this light blue rectangular gift box. Its sophisticated design and decorative bow create perfect packaging for jewellery, accessories, and other special presents, making every occasion memorable. Key features Long rectangular shape is ideal for slim gifts and accessories like watches or pens. Made from durable paper, offering a lightweight and eco-friendly packaging solution. Features an elegant decorative bow, providing a ready-to-gift appearance. Convenient removable lid allows for easy placement and stylish presentation of items. Compact profile ensures easy storage before use and after gifting. Neat light blue finish complements birthdays, anniversaries, and festive occasions. Reusable box can help organise small personal accessories or keep&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="U56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W56" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22311-1-02.jpg</t>
-        </is>
-      </c>
-      <c r="X56" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22311-2-01.jpg</t>
-        </is>
-      </c>
-      <c r="Y56" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22311-3-03.jpg</t>
-        </is>
-      </c>
-      <c r="Z56" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22311-4-04.jpg</t>
-        </is>
-      </c>
-      <c r="AA56" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22311-5-07.jpg</t>
-        </is>
-      </c>
-      <c r="AB56" t="inlineStr">
-        <is>
-          <t>https://cdn.shopify.com/s/files/1/0782/3284/6646/files/22311-6-06.jpg</t>
-        </is>
-      </c>
-    </row>
+    <row r="2" ht="51" customHeight="1"/>
+    <row r="3" ht="51" customHeight="1"/>
+    <row r="4" ht="51" customHeight="1"/>
+    <row r="5" ht="51" customHeight="1"/>
+    <row r="6" ht="51" customHeight="1"/>
+    <row r="7" ht="51" customHeight="1"/>
+    <row r="8" ht="51" customHeight="1"/>
+    <row r="9" ht="51" customHeight="1"/>
+    <row r="10" ht="51" customHeight="1"/>
+    <row r="11" ht="51" customHeight="1"/>
+    <row r="12" ht="51" customHeight="1"/>
+    <row r="13" ht="51" customHeight="1"/>
+    <row r="14" ht="51" customHeight="1"/>
+    <row r="15" ht="51" customHeight="1"/>
+    <row r="16" ht="51" customHeight="1"/>
+    <row r="17" ht="51" customHeight="1"/>
+    <row r="18" ht="51" customHeight="1"/>
+    <row r="19" ht="51" customHeight="1"/>
+    <row r="20" ht="51" customHeight="1"/>
+    <row r="21" ht="51" customHeight="1"/>
+    <row r="22" ht="51" customHeight="1"/>
+    <row r="23" ht="51" customHeight="1"/>
+    <row r="24" ht="51" customHeight="1"/>
+    <row r="25" ht="51" customHeight="1"/>
+    <row r="26" ht="51" customHeight="1"/>
+    <row r="27" ht="51" customHeight="1"/>
+    <row r="28" ht="51" customHeight="1"/>
+    <row r="29" ht="51" customHeight="1"/>
+    <row r="30" ht="51" customHeight="1"/>
+    <row r="31" ht="51" customHeight="1"/>
+    <row r="32" ht="51" customHeight="1"/>
+    <row r="33" ht="51" customHeight="1"/>
+    <row r="34" ht="51" customHeight="1"/>
+    <row r="35" ht="51" customHeight="1"/>
+    <row r="36" ht="51" customHeight="1"/>
+    <row r="37" ht="51" customHeight="1"/>
+    <row r="38" ht="51" customHeight="1"/>
+    <row r="39" ht="51" customHeight="1"/>
+    <row r="40" ht="51" customHeight="1"/>
+    <row r="41" ht="51" customHeight="1"/>
+    <row r="42" ht="51" customHeight="1"/>
+    <row r="43" ht="51" customHeight="1"/>
+    <row r="44" ht="51" customHeight="1"/>
+    <row r="45" ht="51" customHeight="1"/>
+    <row r="46" ht="51" customHeight="1"/>
+    <row r="47" ht="51" customHeight="1"/>
+    <row r="48" ht="51" customHeight="1"/>
+    <row r="49" ht="51" customHeight="1"/>
+    <row r="50" ht="51" customHeight="1"/>
+    <row r="51" ht="51" customHeight="1"/>
+    <row r="52" ht="51" customHeight="1"/>
+    <row r="53" ht="51" customHeight="1"/>
+    <row r="54" ht="51" customHeight="1"/>
+    <row r="55" ht="51" customHeight="1"/>
+    <row r="56" ht="51" customHeight="1"/>
     <row r="57" ht="51" customHeight="1"/>
     <row r="58" ht="51" customHeight="1"/>
     <row r="59" ht="51" customHeight="1"/>

</xml_diff>